<commit_message>
cleanroom: generated 15-scenario input snapshot (A1_Outputs + A2 params + otoole); .txt/Outputs stay gitignored/regenerable
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_A_Calibrated_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_A_Calibrated_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -15370,7 +15370,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="3">
@@ -15411,7 +15411,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="4">
@@ -15452,7 +15452,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="5">
@@ -15493,7 +15493,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="6">
@@ -15534,7 +15534,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="7">
@@ -15575,7 +15575,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="8">
@@ -15698,7 +15698,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="11">
@@ -15739,7 +15739,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="12">
@@ -15780,7 +15780,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="13">
@@ -15821,7 +15821,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="14">
@@ -15862,7 +15862,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="15">
@@ -15903,7 +15903,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="16">
@@ -16026,7 +16026,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="19">
@@ -16067,7 +16067,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="20">
@@ -16108,7 +16108,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="21">
@@ -16149,7 +16149,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="22">
@@ -16190,7 +16190,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="23">
@@ -16231,7 +16231,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="24">
@@ -16354,7 +16354,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="27">
@@ -16395,7 +16395,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="28">
@@ -16436,7 +16436,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="29">
@@ -16477,7 +16477,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="30">
@@ -16518,7 +16518,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="31">
@@ -16559,7 +16559,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="32">
@@ -16682,7 +16682,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="35">
@@ -16723,7 +16723,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="36">
@@ -16764,7 +16764,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="37">
@@ -16805,7 +16805,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="38">
@@ -16846,7 +16846,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="39">
@@ -16887,7 +16887,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="40">
@@ -17010,7 +17010,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="43">
@@ -17051,7 +17051,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="44">
@@ -17092,7 +17092,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="45">
@@ -17133,7 +17133,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="46">
@@ -17174,7 +17174,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="47">
@@ -17215,7 +17215,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="48">
@@ -17338,7 +17338,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="51">
@@ -17379,7 +17379,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="52">
@@ -17420,7 +17420,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="53">
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="54">
@@ -17502,7 +17502,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="55">
@@ -17543,7 +17543,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="56">
@@ -17666,7 +17666,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="59">
@@ -17707,7 +17707,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="60">
@@ -17748,7 +17748,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="61">
@@ -17789,7 +17789,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="62">
@@ -17830,7 +17830,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="63">
@@ -17871,7 +17871,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="64">
@@ -17994,7 +17994,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="67">
@@ -18035,7 +18035,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="68">
@@ -18076,7 +18076,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="69">
@@ -18117,7 +18117,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="70">
@@ -18158,7 +18158,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="71">
@@ -18199,7 +18199,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="72">
@@ -18322,7 +18322,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="75">
@@ -18363,7 +18363,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="76">
@@ -18404,7 +18404,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="77">
@@ -18445,7 +18445,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="78">
@@ -18486,7 +18486,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="79">
@@ -18527,7 +18527,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="80">

</xml_diff>